<commit_message>
Update C0010 data organization and thermal plots
</commit_message>
<xml_diff>
--- a/data/C0016/C0016R00_PARK25_AC_THERM_1D_VAL_comparison.xlsx
+++ b/data/C0016/C0016R00_PARK25_AC_THERM_1D_VAL_comparison.xlsx
@@ -684,16 +684,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>46.80946474562074</v>
+        <v>46.98926959885165</v>
       </c>
       <c r="E10" t="n">
-        <v>47.26602150537639</v>
+        <v>47.47806451612905</v>
       </c>
       <c r="F10" t="n">
         <v>1.861965964330409</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9451011934579573</v>
+        <v>0.9443516895978487</v>
       </c>
     </row>
   </sheetData>
@@ -960,16 +960,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>45.011619231206</v>
+        <v>45.19020230027843</v>
       </c>
       <c r="E10" t="n">
-        <v>47.26602150537639</v>
+        <v>47.47806451612905</v>
       </c>
       <c r="F10" t="n">
-        <v>2.254402274170388</v>
+        <v>2.287862215850623</v>
       </c>
       <c r="G10" t="n">
-        <v>0.8750957325921942</v>
+        <v>0.8795643951983515</v>
       </c>
     </row>
   </sheetData>
@@ -1236,16 +1236,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>48.22409752057484</v>
+        <v>48.40282988617224</v>
       </c>
       <c r="E10" t="n">
-        <v>47.26602150537639</v>
+        <v>47.47806451612905</v>
       </c>
       <c r="F10" t="n">
         <v>3.532040380485341</v>
       </c>
       <c r="G10" t="n">
-        <v>5.217305139855672</v>
+        <v>5.21279247074864</v>
       </c>
     </row>
   </sheetData>
@@ -1315,13 +1315,13 @@
         <v>25.34486290705041</v>
       </c>
       <c r="E2" t="n">
-        <v>25.33279449642493</v>
+        <v>25.34729217663272</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01206841062548136</v>
+        <v>0.002429269582307825</v>
       </c>
       <c r="G2" t="n">
-        <v>5.038593000957743e-05</v>
+        <v>2.355283181993422e-06</v>
       </c>
     </row>
     <row r="3">
@@ -1340,13 +1340,13 @@
         <v>26.92437097147405</v>
       </c>
       <c r="E3" t="n">
-        <v>26.86879272197648</v>
+        <v>26.9377466062569</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05557824949756807</v>
+        <v>0.01337563478285375</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0005087498747126388</v>
+        <v>0.000126030080030309</v>
       </c>
     </row>
     <row r="4">
@@ -1365,13 +1365,13 @@
         <v>29.0325592184592</v>
       </c>
       <c r="E4" t="n">
-        <v>28.95561895168576</v>
+        <v>29.06956040345023</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08491074277665334</v>
+        <v>0.03700118499103056</v>
       </c>
       <c r="G4" t="n">
-        <v>0.006002315484351113</v>
+        <v>0.000902020759527602</v>
       </c>
     </row>
     <row r="5">
@@ -1390,13 +1390,13 @@
         <v>29.05087118059021</v>
       </c>
       <c r="E5" t="n">
-        <v>28.96281346443665</v>
+        <v>29.08456370268814</v>
       </c>
       <c r="F5" t="n">
-        <v>1.022182380268593</v>
+        <v>1.677392666600106</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8141226985027343</v>
+        <v>2.233731975224909</v>
       </c>
     </row>
     <row r="6">
@@ -1415,13 +1415,13 @@
         <v>26.76964316076254</v>
       </c>
       <c r="E6" t="n">
-        <v>27.58171160871424</v>
+        <v>28.26736245570081</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8331424338413278</v>
+        <v>1.517783393763079</v>
       </c>
       <c r="G6" t="n">
-        <v>0.6716269512266513</v>
+        <v>2.264241263656077</v>
       </c>
     </row>
     <row r="7">
@@ -1440,13 +1440,13 @@
         <v>27.14674566298584</v>
       </c>
       <c r="E7" t="n">
-        <v>27.96773668311701</v>
+        <v>28.60905130109842</v>
       </c>
       <c r="F7" t="n">
-        <v>0.8333282779287892</v>
+        <v>1.497529223989364</v>
       </c>
       <c r="G7" t="n">
-        <v>0.655123418531009</v>
+        <v>2.213242845990617</v>
       </c>
     </row>
     <row r="8">
@@ -1465,13 +1465,13 @@
         <v>35.76307723748585</v>
       </c>
       <c r="E8" t="n">
-        <v>36.44315102599818</v>
+        <v>36.94566307336534</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9169333128188804</v>
+        <v>1.461032266475716</v>
       </c>
       <c r="G8" t="n">
-        <v>0.6191211910854584</v>
+        <v>1.724455712266143</v>
       </c>
     </row>
     <row r="9">
@@ -1490,13 +1490,13 @@
         <v>44.80787231440843</v>
       </c>
       <c r="E9" t="n">
-        <v>45.53832896481507</v>
+        <v>46.01752509640811</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7304566504066443</v>
+        <v>1.209652781999679</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4607249405264615</v>
+        <v>1.369030369412058</v>
       </c>
     </row>
     <row r="10">
@@ -1512,16 +1512,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>45.011619231206</v>
+        <v>45.19020230027843</v>
       </c>
       <c r="E10" t="n">
-        <v>45.74667135628272</v>
+        <v>46.43361710451523</v>
       </c>
       <c r="F10" t="n">
-        <v>1.022182380268593</v>
+        <v>1.677392666600106</v>
       </c>
       <c r="G10" t="n">
-        <v>0.6975791821593845</v>
+        <v>1.953469017872455</v>
       </c>
     </row>
   </sheetData>
@@ -1591,13 +1591,13 @@
         <v>25.34487208693474</v>
       </c>
       <c r="E2" t="n">
-        <v>25.33279449642493</v>
+        <v>25.34729217663272</v>
       </c>
       <c r="F2" t="n">
-        <v>0.01207759050981139</v>
+        <v>0.002420089697977801</v>
       </c>
       <c r="G2" t="n">
-        <v>5.03766923977087e-05</v>
+        <v>2.337275896589057e-06</v>
       </c>
     </row>
     <row r="3">
@@ -1616,13 +1616,13 @@
         <v>26.9240579298575</v>
       </c>
       <c r="E3" t="n">
-        <v>26.86879272197648</v>
+        <v>26.9377466062569</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05526520788101763</v>
+        <v>0.01368867639940419</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0005036716563414976</v>
+        <v>0.0001290276296378097</v>
       </c>
     </row>
     <row r="4">
@@ -1641,13 +1641,13 @@
         <v>29.03300703192411</v>
       </c>
       <c r="E4" t="n">
-        <v>28.95561895168576</v>
+        <v>29.06956040345023</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08458123546395413</v>
+        <v>0.03655337152611438</v>
       </c>
       <c r="G4" t="n">
-        <v>0.005937659518467908</v>
+        <v>0.0009243437568763117</v>
       </c>
     </row>
     <row r="5">
@@ -1666,13 +1666,13 @@
         <v>30.3869544580445</v>
       </c>
       <c r="E5" t="n">
-        <v>29.90399071228493</v>
+        <v>30.34591953619899</v>
       </c>
       <c r="F5" t="n">
-        <v>0.5237215763559178</v>
+        <v>0.1740708984831407</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1846995175069001</v>
+        <v>0.01117636651837496</v>
       </c>
     </row>
     <row r="6">
@@ -1691,13 +1691,13 @@
         <v>30.25779059894091</v>
       </c>
       <c r="E6" t="n">
-        <v>29.7415513101022</v>
+        <v>30.30371777849071</v>
       </c>
       <c r="F6" t="n">
-        <v>0.5405069270245804</v>
+        <v>0.04592717954979619</v>
       </c>
       <c r="G6" t="n">
-        <v>0.2786217012489927</v>
+        <v>0.001201623331275293</v>
       </c>
     </row>
     <row r="7">
@@ -1716,13 +1716,13 @@
         <v>30.58265939396995</v>
       </c>
       <c r="E7" t="n">
-        <v>30.12757638450496</v>
+        <v>30.64540662388833</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5159119023071383</v>
+        <v>0.06984261838260863</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2461315589779256</v>
+        <v>0.003537799366334877</v>
       </c>
     </row>
     <row r="8">
@@ -1741,13 +1741,13 @@
         <v>39.05463468004791</v>
       </c>
       <c r="E8" t="n">
-        <v>38.60299072738614</v>
+        <v>38.98201839615525</v>
       </c>
       <c r="F8" t="n">
-        <v>0.455035160095715</v>
+        <v>0.07261628389266406</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1728783315952969</v>
+        <v>0.002101141368345586</v>
       </c>
     </row>
     <row r="9">
@@ -1766,13 +1766,13 @@
         <v>48.0201598232307</v>
       </c>
       <c r="E9" t="n">
-        <v>47.69816866620303</v>
+        <v>48.05388041919802</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4517915303931943</v>
+        <v>0.07392394858168672</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1663287087626613</v>
+        <v>0.002601968853802898</v>
       </c>
     </row>
     <row r="10">
@@ -1788,16 +1788,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>48.22409752057484</v>
+        <v>48.40282988617224</v>
       </c>
       <c r="E10" t="n">
-        <v>47.90651105767068</v>
+        <v>48.46997242730514</v>
       </c>
       <c r="F10" t="n">
-        <v>0.5405069270245804</v>
+        <v>0.1740708984831407</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1725137566392716</v>
+        <v>0.008550768373096084</v>
       </c>
     </row>
   </sheetData>
@@ -1864,7 +1864,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>25.33279449642493</v>
+        <v>25.34729217663272</v>
       </c>
       <c r="E2" t="n">
         <v>25.50333333333333</v>
@@ -1873,7 +1873,7 @@
         <v>0.2699999999999818</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04710864037097589</v>
+        <v>0.04753869203839175</v>
       </c>
     </row>
     <row r="3">
@@ -1889,16 +1889,16 @@
         <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>26.86879272197648</v>
+        <v>26.9377466062569</v>
       </c>
       <c r="E3" t="n">
         <v>26.90333333333336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1668880338280907</v>
+        <v>0.1309816741744712</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01025985767758122</v>
+        <v>0.005630114628140404</v>
       </c>
     </row>
     <row r="4">
@@ -1914,16 +1914,16 @@
         <v>180</v>
       </c>
       <c r="D4" t="n">
-        <v>28.95561895168576</v>
+        <v>29.06956040345023</v>
       </c>
       <c r="E4" t="n">
         <v>29.08506944444446</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1294504927586964</v>
+        <v>0.04100563069677321</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01144964255662027</v>
+        <v>0.0002858988701365468</v>
       </c>
     </row>
     <row r="5">
@@ -1939,16 +1939,16 @@
         <v>1560</v>
       </c>
       <c r="D5" t="n">
-        <v>28.96281346443665</v>
+        <v>29.08456370268814</v>
       </c>
       <c r="E5" t="n">
         <v>29.10000000000002</v>
       </c>
       <c r="F5" t="n">
-        <v>0.846228603197968</v>
+        <v>1.52129845610644</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1611695546059887</v>
+        <v>0.6921114262084015</v>
       </c>
     </row>
     <row r="6">
@@ -1964,16 +1964,16 @@
         <v>1632</v>
       </c>
       <c r="D6" t="n">
-        <v>27.58171160871424</v>
+        <v>28.26736245570081</v>
       </c>
       <c r="E6" t="n">
         <v>27.34083333333336</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8379796336776728</v>
+        <v>1.522620593599424</v>
       </c>
       <c r="G6" t="n">
-        <v>0.320581591558486</v>
+        <v>1.528774548916671</v>
       </c>
     </row>
     <row r="7">
@@ -1989,16 +1989,16 @@
         <v>1719</v>
       </c>
       <c r="D7" t="n">
-        <v>27.96773668311701</v>
+        <v>28.60905130109842</v>
       </c>
       <c r="E7" t="n">
         <v>27.68609195402297</v>
       </c>
       <c r="F7" t="n">
-        <v>0.2816447290940403</v>
+        <v>0.9229593470754516</v>
       </c>
       <c r="G7" t="n">
-        <v>0.01990814653990782</v>
+        <v>0.6442099238612781</v>
       </c>
     </row>
     <row r="8">
@@ -2014,16 +2014,16 @@
         <v>1824</v>
       </c>
       <c r="D8" t="n">
-        <v>36.44315102599818</v>
+        <v>36.94566307336534</v>
       </c>
       <c r="E8" t="n">
         <v>37.20847619047618</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7685228558564248</v>
+        <v>0.9417992788309313</v>
       </c>
       <c r="G8" t="n">
-        <v>0.4385686604235871</v>
+        <v>0.07800114326204935</v>
       </c>
     </row>
     <row r="9">
@@ -2039,16 +2039,16 @@
         <v>1917</v>
       </c>
       <c r="D9" t="n">
-        <v>45.53832896481507</v>
+        <v>46.01752509640811</v>
       </c>
       <c r="E9" t="n">
         <v>47.05397849462366</v>
       </c>
       <c r="F9" t="n">
-        <v>1.515649529808591</v>
+        <v>1.036453398215556</v>
       </c>
       <c r="G9" t="n">
-        <v>1.559349335545858</v>
+        <v>0.5965118396320634</v>
       </c>
     </row>
     <row r="10">
@@ -2064,16 +2064,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>45.74667135628272</v>
+        <v>46.43361710451523</v>
       </c>
       <c r="E10" t="n">
-        <v>47.26602150537639</v>
+        <v>47.47806451612905</v>
       </c>
       <c r="F10" t="n">
-        <v>1.519350149093668</v>
+        <v>1.522620593599424</v>
       </c>
       <c r="G10" t="n">
-        <v>0.2319685870382768</v>
+        <v>0.619329961900869</v>
       </c>
     </row>
   </sheetData>
@@ -2140,7 +2140,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="n">
-        <v>25.33279449642493</v>
+        <v>25.34729217663272</v>
       </c>
       <c r="E2" t="n">
         <v>25.50333333333333</v>
@@ -2149,7 +2149,7 @@
         <v>0.2699999999999818</v>
       </c>
       <c r="G2" t="n">
-        <v>0.04710864037097589</v>
+        <v>0.04753869203839175</v>
       </c>
     </row>
     <row r="3">
@@ -2165,16 +2165,16 @@
         <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>26.86879272197648</v>
+        <v>26.9377466062569</v>
       </c>
       <c r="E3" t="n">
         <v>26.90333333333336</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1668880338280907</v>
+        <v>0.1309816741744712</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01025985767758122</v>
+        <v>0.005630114628140404</v>
       </c>
     </row>
     <row r="4">
@@ -2190,16 +2190,16 @@
         <v>180</v>
       </c>
       <c r="D4" t="n">
-        <v>28.95561895168576</v>
+        <v>29.06956040345023</v>
       </c>
       <c r="E4" t="n">
         <v>29.08506944444446</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1294504927586964</v>
+        <v>0.04100563069677321</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01144964255662027</v>
+        <v>0.0002858988701365468</v>
       </c>
     </row>
     <row r="5">
@@ -2215,16 +2215,16 @@
         <v>1560</v>
       </c>
       <c r="D5" t="n">
-        <v>29.90399071228493</v>
+        <v>30.34591953619899</v>
       </c>
       <c r="E5" t="n">
         <v>29.10000000000002</v>
       </c>
       <c r="F5" t="n">
-        <v>3.00642507095781</v>
+        <v>3.557415875611539</v>
       </c>
       <c r="G5" t="n">
-        <v>3.970134156834253</v>
+        <v>5.575137709435875</v>
       </c>
     </row>
     <row r="6">
@@ -2240,16 +2240,16 @@
         <v>1632</v>
       </c>
       <c r="D6" t="n">
-        <v>29.7415513101022</v>
+        <v>30.30371777849071</v>
       </c>
       <c r="E6" t="n">
         <v>27.34083333333336</v>
       </c>
       <c r="F6" t="n">
-        <v>2.997947515721421</v>
+        <v>3.558860290705123</v>
       </c>
       <c r="G6" t="n">
-        <v>7.314162976588908</v>
+        <v>10.66172654431028</v>
       </c>
     </row>
     <row r="7">
@@ -2265,16 +2265,16 @@
         <v>1719</v>
       </c>
       <c r="D7" t="n">
-        <v>30.12757638450496</v>
+        <v>30.64540662388833</v>
       </c>
       <c r="E7" t="n">
         <v>27.68609195402297</v>
       </c>
       <c r="F7" t="n">
-        <v>2.441484430481989</v>
+        <v>2.959314669865361</v>
       </c>
       <c r="G7" t="n">
-        <v>5.208247495264174</v>
+        <v>8.047089062915122</v>
       </c>
     </row>
     <row r="8">
@@ -2290,16 +2290,16 @@
         <v>1824</v>
       </c>
       <c r="D8" t="n">
-        <v>38.60299072738614</v>
+        <v>38.98201839615525</v>
       </c>
       <c r="E8" t="n">
         <v>37.20847619047618</v>
       </c>
       <c r="F8" t="n">
-        <v>2.460589403516604</v>
+        <v>2.978154601620844</v>
       </c>
       <c r="G8" t="n">
-        <v>2.407914918343024</v>
+        <v>3.826234499686215</v>
       </c>
     </row>
     <row r="9">
@@ -2315,16 +2315,16 @@
         <v>1917</v>
       </c>
       <c r="D9" t="n">
-        <v>47.69816866620303</v>
+        <v>48.05388041919802</v>
       </c>
       <c r="E9" t="n">
         <v>47.05397849462366</v>
       </c>
       <c r="F9" t="n">
-        <v>1.39535714431657</v>
+        <v>1.774185604924028</v>
       </c>
       <c r="G9" t="n">
-        <v>0.91823789200115</v>
+        <v>1.742236650917256</v>
       </c>
     </row>
     <row r="10">
@@ -2340,16 +2340,16 @@
         <v>1917</v>
       </c>
       <c r="D10" t="n">
-        <v>47.90651105767068</v>
+        <v>48.46997242730514</v>
       </c>
       <c r="E10" t="n">
-        <v>47.26602150537639</v>
+        <v>47.47806451612905</v>
       </c>
       <c r="F10" t="n">
-        <v>3.00642507095781</v>
+        <v>3.558860290705123</v>
       </c>
       <c r="G10" t="n">
-        <v>3.54341402877584</v>
+        <v>5.064896891277852</v>
       </c>
     </row>
   </sheetData>

</xml_diff>